<commit_message>
feat: optimizar sistema de exportación y generación de reportes
</commit_message>
<xml_diff>
--- a/templates/reporte_base.xlsx
+++ b/templates/reporte_base.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Neisa S\Documents\SISTEMA_CONTROL_DE_CUENTA\templates\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6ADD4202-333D-47D4-B303-02577412FA3A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4ABD97DC-1B6E-466B-B749-D50AA2F17750}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="24" yWindow="384" windowWidth="23016" windowHeight="12216" xr2:uid="{B67AD9E5-769A-4932-96AF-B3196C137F9D}"/>
+    <workbookView xWindow="12" yWindow="12" windowWidth="23016" windowHeight="12216" xr2:uid="{B67AD9E5-769A-4932-96AF-B3196C137F9D}"/>
   </bookViews>
   <sheets>
     <sheet name="Hoja1" sheetId="1" r:id="rId1"/>
@@ -40,7 +40,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="20" uniqueCount="17">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="19" uniqueCount="17">
   <si>
     <t xml:space="preserve"> </t>
   </si>
@@ -791,7 +791,7 @@
     <xf numFmtId="0" fontId="8" fillId="2" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="8" fillId="2" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="49" fontId="8" fillId="2" borderId="8" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="4" fillId="2" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -824,59 +824,59 @@
     <xf numFmtId="164" fontId="7" fillId="7" borderId="23" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="24" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="25" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="28" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="2" fillId="7" borderId="30" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="2" fillId="7" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="2" fillId="7" borderId="31" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="2" fillId="7" borderId="32" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="7" borderId="26" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="7" borderId="27" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="7" borderId="9" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="7" borderId="10" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="3" borderId="33" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="3" borderId="34" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="1" fillId="3" borderId="31" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
+      <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="3" borderId="32" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="3" borderId="24" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="3" borderId="25" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="3" borderId="28" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="3" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="164" fontId="2" fillId="7" borderId="30" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="164" fontId="2" fillId="7" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="164" fontId="2" fillId="7" borderId="31" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="164" fontId="2" fillId="7" borderId="32" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="7" borderId="26" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="7" borderId="27" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="7" borderId="9" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="7" borderId="10" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="3" borderId="33" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="3" borderId="34" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
+      <alignment vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -1226,7 +1226,7 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{B99FB1B7-8980-4948-B759-79414B110038}">
   <sheetPr codeName="Hoja1"/>
-  <dimension ref="A1:K36"/>
+  <dimension ref="A1:J20"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="11.5546875" style="1" customWidth="1"/>
@@ -1286,67 +1286,61 @@
       <c r="F5" s="13"/>
       <c r="G5" s="13"/>
       <c r="H5" s="12"/>
-      <c r="J5" s="49"/>
+      <c r="J5" s="47"/>
     </row>
     <row r="6" spans="1:10" ht="14.4" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B6" s="11"/>
-      <c r="C6" s="51" t="s">
+      <c r="C6" s="49" t="s">
         <v>10</v>
       </c>
-      <c r="D6" s="52"/>
-      <c r="E6" s="59" t="s">
+      <c r="D6" s="50"/>
+      <c r="E6" s="57" t="s">
         <v>1</v>
       </c>
-      <c r="F6" s="60"/>
+      <c r="F6" s="58"/>
       <c r="G6" s="23"/>
       <c r="H6" s="12"/>
-      <c r="J6" s="49"/>
+      <c r="J6" s="47"/>
     </row>
     <row r="7" spans="1:10" ht="14.4" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B7" s="11"/>
-      <c r="C7" s="53"/>
-      <c r="D7" s="54"/>
-      <c r="E7" s="61" t="s">
+      <c r="C7" s="51"/>
+      <c r="D7" s="52"/>
+      <c r="E7" s="59" t="s">
         <v>2</v>
       </c>
-      <c r="F7" s="62"/>
-      <c r="G7" s="24">
-        <f>SUM(E15:E33)</f>
-        <v>0</v>
-      </c>
+      <c r="F7" s="60"/>
+      <c r="G7" s="24"/>
       <c r="H7" s="12"/>
     </row>
     <row r="8" spans="1:10" ht="14.4" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B8" s="11"/>
-      <c r="C8" s="55" t="s">
+      <c r="C8" s="53" t="s">
         <v>5</v>
       </c>
-      <c r="D8" s="56"/>
-      <c r="E8" s="61" t="s">
+      <c r="D8" s="54"/>
+      <c r="E8" s="59" t="s">
         <v>3</v>
       </c>
-      <c r="F8" s="62"/>
-      <c r="G8" s="24">
-        <f>SUM(F15:F33)</f>
-        <v>0</v>
-      </c>
+      <c r="F8" s="60"/>
+      <c r="G8" s="24"/>
       <c r="H8" s="12"/>
-      <c r="J8" s="50"/>
+      <c r="J8" s="48"/>
     </row>
     <row r="9" spans="1:10" ht="14.4" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
       <c r="B9" s="11"/>
-      <c r="C9" s="57"/>
-      <c r="D9" s="58"/>
-      <c r="E9" s="63" t="s">
+      <c r="C9" s="55"/>
+      <c r="D9" s="56"/>
+      <c r="E9" s="61" t="s">
         <v>4</v>
       </c>
-      <c r="F9" s="64"/>
+      <c r="F9" s="62"/>
       <c r="G9" s="25">
         <f>G6+G7-G8</f>
         <v>0</v>
       </c>
       <c r="H9" s="12"/>
-      <c r="J9" s="50"/>
+      <c r="J9" s="48"/>
     </row>
     <row r="10" spans="1:10" ht="14.4" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
       <c r="B10" s="11"/>
@@ -1426,259 +1420,57 @@
     </row>
     <row r="16" spans="1:10" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B16" s="11"/>
-      <c r="C16" s="29"/>
+      <c r="C16" s="31"/>
       <c r="D16" s="2"/>
       <c r="E16" s="3"/>
       <c r="F16" s="4"/>
-      <c r="G16" s="30">
-        <f>G15+E16-F16</f>
+      <c r="G16" s="30"/>
+      <c r="H16" s="12"/>
+    </row>
+    <row r="17" spans="2:8" ht="15" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="B17" s="11"/>
+      <c r="C17" s="32"/>
+      <c r="D17" s="5"/>
+      <c r="E17" s="6"/>
+      <c r="F17" s="7"/>
+      <c r="G17" s="30"/>
+      <c r="H17" s="12"/>
+    </row>
+    <row r="18" spans="2:8" ht="19.8" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="B18" s="11"/>
+      <c r="C18" s="63" t="s">
+        <v>12</v>
+      </c>
+      <c r="D18" s="64"/>
+      <c r="E18" s="33">
+        <f>SUM(E15:E17)</f>
         <v>0</v>
       </c>
-      <c r="H16" s="12"/>
-    </row>
-    <row r="17" spans="2:11" ht="15" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B17" s="11"/>
-      <c r="C17" s="31"/>
-      <c r="D17" s="2"/>
-      <c r="E17" s="3"/>
-      <c r="F17" s="4"/>
-      <c r="G17" s="30">
-        <f t="shared" ref="G17:G33" si="0">G16+E17-F17</f>
+      <c r="F18" s="33">
+        <f>SUM(F15:F17)</f>
         <v>0</v>
       </c>
-      <c r="H17" s="12"/>
-    </row>
-    <row r="18" spans="2:11" ht="15" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B18" s="11"/>
-      <c r="C18" s="31"/>
-      <c r="D18" s="2"/>
-      <c r="E18" s="3"/>
-      <c r="F18" s="4"/>
-      <c r="G18" s="30">
-        <f t="shared" si="0"/>
+      <c r="G18" s="34">
+        <f>E18-F18</f>
         <v>0</v>
       </c>
       <c r="H18" s="12"/>
     </row>
-    <row r="19" spans="2:11" ht="15" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B19" s="11"/>
-      <c r="C19" s="31"/>
-      <c r="D19" s="2"/>
-      <c r="E19" s="3"/>
-      <c r="F19" s="4"/>
-      <c r="G19" s="30">
-        <f t="shared" si="0"/>
-        <v>0</v>
-      </c>
-      <c r="H19" s="12"/>
-      <c r="K19" s="1" t="s">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="20" spans="2:11" ht="15" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B20" s="11"/>
-      <c r="C20" s="29"/>
-      <c r="D20" s="2"/>
-      <c r="E20" s="3"/>
-      <c r="F20" s="4"/>
-      <c r="G20" s="30">
-        <f t="shared" si="0"/>
-        <v>0</v>
-      </c>
-      <c r="H20" s="12"/>
-    </row>
-    <row r="21" spans="2:11" ht="15" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B21" s="11"/>
-      <c r="C21" s="29"/>
-      <c r="D21" s="2"/>
-      <c r="E21" s="3"/>
-      <c r="F21" s="4"/>
-      <c r="G21" s="30">
-        <f t="shared" si="0"/>
-        <v>0</v>
-      </c>
-      <c r="H21" s="12"/>
-    </row>
-    <row r="22" spans="2:11" ht="15" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B22" s="11"/>
-      <c r="C22" s="29"/>
-      <c r="D22" s="2"/>
-      <c r="E22" s="3"/>
-      <c r="F22" s="4"/>
-      <c r="G22" s="30">
-        <f t="shared" si="0"/>
-        <v>0</v>
-      </c>
-      <c r="H22" s="12"/>
-    </row>
-    <row r="23" spans="2:11" ht="15" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B23" s="11"/>
-      <c r="C23" s="29"/>
-      <c r="D23" s="2"/>
-      <c r="E23" s="3"/>
-      <c r="F23" s="4"/>
-      <c r="G23" s="30">
-        <f t="shared" si="0"/>
-        <v>0</v>
-      </c>
-      <c r="H23" s="12"/>
-    </row>
-    <row r="24" spans="2:11" ht="15" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B24" s="11"/>
-      <c r="C24" s="29"/>
-      <c r="D24" s="2"/>
-      <c r="E24" s="3"/>
-      <c r="F24" s="4"/>
-      <c r="G24" s="30">
-        <f t="shared" si="0"/>
-        <v>0</v>
-      </c>
-      <c r="H24" s="12"/>
-    </row>
-    <row r="25" spans="2:11" ht="15" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B25" s="11"/>
-      <c r="C25" s="29"/>
-      <c r="D25" s="2"/>
-      <c r="E25" s="3"/>
-      <c r="F25" s="4"/>
-      <c r="G25" s="30">
-        <f t="shared" si="0"/>
-        <v>0</v>
-      </c>
-      <c r="H25" s="12"/>
-    </row>
-    <row r="26" spans="2:11" ht="15" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B26" s="11"/>
-      <c r="C26" s="29"/>
-      <c r="D26" s="2"/>
-      <c r="E26" s="3"/>
-      <c r="F26" s="4"/>
-      <c r="G26" s="30">
-        <f t="shared" si="0"/>
-        <v>0</v>
-      </c>
-      <c r="H26" s="12"/>
-    </row>
-    <row r="27" spans="2:11" ht="15" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B27" s="11"/>
-      <c r="C27" s="29"/>
-      <c r="D27" s="2"/>
-      <c r="E27" s="3"/>
-      <c r="F27" s="4"/>
-      <c r="G27" s="30">
-        <f t="shared" si="0"/>
-        <v>0</v>
-      </c>
-      <c r="H27" s="12"/>
-    </row>
-    <row r="28" spans="2:11" ht="15" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B28" s="11"/>
-      <c r="C28" s="29"/>
-      <c r="D28" s="2"/>
-      <c r="E28" s="3"/>
-      <c r="F28" s="4"/>
-      <c r="G28" s="30">
-        <f t="shared" si="0"/>
-        <v>0</v>
-      </c>
-      <c r="H28" s="12"/>
-    </row>
-    <row r="29" spans="2:11" ht="15" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B29" s="11"/>
-      <c r="C29" s="29"/>
-      <c r="D29" s="2"/>
-      <c r="E29" s="3"/>
-      <c r="F29" s="4"/>
-      <c r="G29" s="30">
-        <f t="shared" si="0"/>
-        <v>0</v>
-      </c>
-      <c r="H29" s="12"/>
-    </row>
-    <row r="30" spans="2:11" ht="15" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B30" s="11"/>
-      <c r="C30" s="29"/>
-      <c r="D30" s="2"/>
-      <c r="E30" s="3"/>
-      <c r="F30" s="4"/>
-      <c r="G30" s="30">
-        <f t="shared" si="0"/>
-        <v>0</v>
-      </c>
-      <c r="H30" s="12"/>
-    </row>
-    <row r="31" spans="2:11" ht="15" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B31" s="11"/>
-      <c r="C31" s="29"/>
-      <c r="D31" s="2"/>
-      <c r="E31" s="3"/>
-      <c r="F31" s="4"/>
-      <c r="G31" s="30">
-        <f t="shared" si="0"/>
-        <v>0</v>
-      </c>
-      <c r="H31" s="12"/>
-    </row>
-    <row r="32" spans="2:11" ht="15" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B32" s="11"/>
-      <c r="C32" s="29"/>
-      <c r="D32" s="2"/>
-      <c r="E32" s="3"/>
-      <c r="F32" s="4"/>
-      <c r="G32" s="30">
-        <f t="shared" si="0"/>
-        <v>0</v>
-      </c>
-      <c r="H32" s="12"/>
-    </row>
-    <row r="33" spans="2:8" ht="15" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="B33" s="11"/>
-      <c r="C33" s="32"/>
-      <c r="D33" s="5"/>
-      <c r="E33" s="6"/>
-      <c r="F33" s="7"/>
-      <c r="G33" s="30">
-        <f t="shared" si="0"/>
-        <v>0</v>
-      </c>
-      <c r="H33" s="12"/>
-    </row>
-    <row r="34" spans="2:8" ht="19.8" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="B34" s="11"/>
-      <c r="C34" s="47" t="s">
-        <v>12</v>
-      </c>
-      <c r="D34" s="48"/>
-      <c r="E34" s="33">
-        <f>SUM(E15:E33)</f>
-        <v>0</v>
-      </c>
-      <c r="F34" s="33">
-        <f>SUM(F15:F33)</f>
-        <v>0</v>
-      </c>
-      <c r="G34" s="34">
-        <f>E34-F34</f>
-        <v>0</v>
-      </c>
-      <c r="H34" s="12"/>
-    </row>
-    <row r="35" spans="2:8" ht="15" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="B35" s="15"/>
-      <c r="C35" s="16"/>
-      <c r="D35" s="16"/>
-      <c r="E35" s="16"/>
-      <c r="F35" s="16"/>
-      <c r="G35" s="16"/>
-      <c r="H35" s="14"/>
-    </row>
-    <row r="36" spans="2:8" ht="15" thickTop="1" x14ac:dyDescent="0.3"/>
+    <row r="19" spans="2:8" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="B19" s="15"/>
+      <c r="C19" s="16"/>
+      <c r="D19" s="16"/>
+      <c r="E19" s="16"/>
+      <c r="F19" s="16"/>
+      <c r="G19" s="16"/>
+      <c r="H19" s="14"/>
+    </row>
+    <row r="20" spans="2:8" ht="15" thickTop="1" x14ac:dyDescent="0.3"/>
   </sheetData>
-  <mergeCells count="12">
+  <mergeCells count="11">
     <mergeCell ref="C3:E4"/>
     <mergeCell ref="C11:G11"/>
     <mergeCell ref="C12:G12"/>
-    <mergeCell ref="C34:D34"/>
     <mergeCell ref="J5:J6"/>
     <mergeCell ref="J8:J9"/>
     <mergeCell ref="C6:D7"/>

</xml_diff>